<commit_message>
only show high coverage weights by risk
</commit_message>
<xml_diff>
--- a/data/inputs/sample_scenario.xlsx
+++ b/data/inputs/sample_scenario.xlsx
@@ -36,8 +36,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="0.0%;[Red]\ \-0.0%;\ 0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -431,71 +434,71 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>US Equity</v>
+        <v>Cash</v>
       </c>
       <c r="B2" t="str">
-        <v>0.075</v>
+        <v>0.0360</v>
       </c>
       <c r="C2" t="str">
-        <v>0.18</v>
+        <v>0.0020</v>
       </c>
       <c r="D2" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="G2" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="H2" t="str">
         <v>0</v>
-      </c>
-      <c r="E2" t="str">
-        <v>0.6</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Equity</v>
-      </c>
-      <c r="G2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H2" t="str">
-        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Dev ex-US Equity</v>
+        <v>Government Bonds</v>
       </c>
       <c r="B3" t="str">
-        <v>0.065</v>
+        <v>0.0420</v>
       </c>
       <c r="C3" t="str">
-        <v>0.16</v>
+        <v>0.0550</v>
       </c>
       <c r="D3" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="E3" t="str">
+        <v>0.075</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Fixed Income</v>
+      </c>
+      <c r="G3" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="H3" t="str">
         <v>0</v>
-      </c>
-      <c r="E3" t="str">
-        <v>0.6</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Equity</v>
-      </c>
-      <c r="G3" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H3" t="str">
-        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Emerging Equity</v>
+        <v>Global Equities (Passive)</v>
       </c>
       <c r="B4" t="str">
-        <v>0.085</v>
+        <v>0.0600</v>
       </c>
       <c r="C4" t="str">
-        <v>0.22</v>
+        <v>0.1600</v>
       </c>
       <c r="D4" t="str">
-        <v>0</v>
+        <v>0.00</v>
       </c>
       <c r="E4" t="str">
-        <v>0.4</v>
+        <v>1.00</v>
       </c>
       <c r="F4" t="str">
         <v>Equity</v>
@@ -504,85 +507,85 @@
         <v>USD</v>
       </c>
       <c r="H4" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Global IG Bonds</v>
+        <v>Private Equity</v>
       </c>
       <c r="B5" t="str">
-        <v>0.025</v>
+        <v>0.1100</v>
       </c>
       <c r="C5" t="str">
-        <v>0.06</v>
+        <v>0.2000</v>
       </c>
       <c r="D5" t="str">
-        <v>0.1</v>
+        <v>0.00</v>
       </c>
       <c r="E5" t="str">
-        <v>0.8</v>
+        <v>0.25</v>
       </c>
       <c r="F5" t="str">
-        <v>Fixed Income</v>
+        <v>Illiquid</v>
       </c>
       <c r="G5" t="str">
         <v>USD</v>
       </c>
       <c r="H5" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EM Debt (HC)</v>
+        <v>Inflation Linked Bonds</v>
       </c>
       <c r="B6" t="str">
-        <v>0.04</v>
+        <v>0.0420</v>
       </c>
       <c r="C6" t="str">
-        <v>0.1</v>
+        <v>0.0550</v>
       </c>
       <c r="D6" t="str">
-        <v>0</v>
+        <v>0.00</v>
       </c>
       <c r="E6" t="str">
-        <v>0.3</v>
+        <v>0.075</v>
       </c>
       <c r="F6" t="str">
         <v>Fixed Income</v>
       </c>
       <c r="G6" t="str">
-        <v>USD</v>
+        <v>GBP</v>
       </c>
       <c r="H6" t="str">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Global REITs</v>
+        <v>Multi-asset class</v>
       </c>
       <c r="B7" t="str">
-        <v>0.06</v>
+        <v>0.0740</v>
       </c>
       <c r="C7" t="str">
-        <v>0.18</v>
+        <v>0.0861</v>
       </c>
       <c r="D7" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="E7" t="str">
+        <v>1.00</v>
+      </c>
+      <c r="F7" t="str">
+        <v>MAC</v>
+      </c>
+      <c r="G7" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="H7" t="str">
         <v>0</v>
-      </c>
-      <c r="E7" t="str">
-        <v>0.3</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Real Assets</v>
-      </c>
-      <c r="G7" t="str">
-        <v>USD</v>
-      </c>
-      <c r="H7" t="str">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -601,160 +604,160 @@
         <v>Asset</v>
       </c>
       <c r="B1" t="str">
-        <v>US Equity</v>
+        <v>Cash</v>
       </c>
       <c r="C1" t="str">
-        <v>Dev ex-US Equity</v>
+        <v>Government Bonds</v>
       </c>
       <c r="D1" t="str">
-        <v>Emerging Equity</v>
+        <v>Global Equities (Passive)</v>
       </c>
       <c r="E1" t="str">
-        <v>Global IG Bonds</v>
+        <v>Private Equity</v>
       </c>
       <c r="F1" t="str">
-        <v>EM Debt (HC)</v>
+        <v>Inflation Linked Bonds</v>
       </c>
       <c r="G1" t="str">
-        <v>Global REITs</v>
+        <v>Multi-asset class</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>US Equity</v>
+        <v>Cash</v>
       </c>
       <c r="B2" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
       <c r="C2" t="str">
-        <v>0.8</v>
+        <v xml:space="preserve">0.18 </v>
       </c>
       <c r="D2" t="str">
-        <v>0.75</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="E2" t="str">
-        <v>0.2</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="F2" t="str">
-        <v>0.35</v>
+        <v xml:space="preserve">0.09 </v>
       </c>
       <c r="G2" t="str">
-        <v>0.6</v>
+        <v xml:space="preserve">0.08 </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Dev ex-US Equity</v>
+        <v>Government Bonds</v>
       </c>
       <c r="B3" t="str">
-        <v>0.8</v>
+        <v xml:space="preserve">0.18 </v>
       </c>
       <c r="C3" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
       <c r="D3" t="str">
-        <v>0.78</v>
+        <v xml:space="preserve">0.01 </v>
       </c>
       <c r="E3" t="str">
-        <v>0.18</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="F3" t="str">
-        <v>0.32</v>
+        <v xml:space="preserve">0.48 </v>
       </c>
       <c r="G3" t="str">
-        <v>0.58</v>
+        <v xml:space="preserve">0.40 </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Emerging Equity</v>
+        <v>Global Equities (Passive)</v>
       </c>
       <c r="B4" t="str">
-        <v>0.75</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="C4" t="str">
-        <v>0.78</v>
+        <v xml:space="preserve">0.01 </v>
       </c>
       <c r="D4" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
       <c r="E4" t="str">
-        <v>0.15</v>
+        <v xml:space="preserve">0.71 </v>
       </c>
       <c r="F4" t="str">
-        <v>0.3</v>
+        <v xml:space="preserve">0.02 </v>
       </c>
       <c r="G4" t="str">
-        <v>0.55</v>
+        <v xml:space="preserve">0.60 </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Global IG Bonds</v>
+        <v>Private Equity</v>
       </c>
       <c r="B5" t="str">
-        <v>0.2</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="C5" t="str">
-        <v>0.18</v>
+        <v xml:space="preserve">0.00 </v>
       </c>
       <c r="D5" t="str">
-        <v>0.15</v>
+        <v xml:space="preserve">0.71 </v>
       </c>
       <c r="E5" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
       <c r="F5" t="str">
-        <v>0.3</v>
+        <v>0.00</v>
       </c>
       <c r="G5" t="str">
-        <v>0.25</v>
+        <v xml:space="preserve">0.48 </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EM Debt (HC)</v>
+        <v>Inflation Linked Bonds</v>
       </c>
       <c r="B6" t="str">
-        <v>0.35</v>
+        <v xml:space="preserve">0.09 </v>
       </c>
       <c r="C6" t="str">
-        <v>0.32</v>
+        <v xml:space="preserve">0.48 </v>
       </c>
       <c r="D6" t="str">
-        <v>0.3</v>
+        <v xml:space="preserve">0.02 </v>
       </c>
       <c r="E6" t="str">
-        <v>0.3</v>
+        <v>0.00</v>
       </c>
       <c r="F6" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
       <c r="G6" t="str">
-        <v>0.4</v>
+        <v xml:space="preserve">0.20 </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Global REITs</v>
+        <v>Multi-asset class</v>
       </c>
       <c r="B7" t="str">
-        <v>0.6</v>
+        <v xml:space="preserve">0.08 </v>
       </c>
       <c r="C7" t="str">
-        <v>0.58</v>
+        <v xml:space="preserve">0.40 </v>
       </c>
       <c r="D7" t="str">
-        <v>0.55</v>
+        <v xml:space="preserve">0.60 </v>
       </c>
       <c r="E7" t="str">
-        <v>0.25</v>
+        <v xml:space="preserve">0.48 </v>
       </c>
       <c r="F7" t="str">
-        <v>0.4</v>
+        <v xml:space="preserve">0.20 </v>
       </c>
       <c r="G7" t="str">
-        <v>1</v>
+        <v xml:space="preserve">1.00 </v>
       </c>
     </row>
   </sheetData>
@@ -781,7 +784,7 @@
         <v>RiskFreeRate</v>
       </c>
       <c r="B2" t="str">
-        <v>0</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="3">
@@ -821,7 +824,7 @@
         <v>Resamples</v>
       </c>
       <c r="B7" t="str">
-        <v>400</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -829,7 +832,7 @@
         <v>ResampleYears</v>
       </c>
       <c r="B8" t="str">
-        <v>40</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -899,7 +902,7 @@
         <v>HorizonYears</v>
       </c>
       <c r="B2" t="str">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -907,7 +910,7 @@
         <v>NumPaths</v>
       </c>
       <c r="B3" t="str">
-        <v>10000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4">
@@ -915,7 +918,7 @@
         <v>StartWealth</v>
       </c>
       <c r="B4" t="str">
-        <v>1000000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="5">
@@ -923,7 +926,7 @@
         <v>InflationRate</v>
       </c>
       <c r="B5" t="str">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="6">
@@ -931,7 +934,7 @@
         <v>StartSpendingYear</v>
       </c>
       <c r="B6" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -1059,7 +1062,7 @@
         <v>ConstantReal</v>
       </c>
       <c r="B2" t="str">
-        <v>40000</v>
+        <v>250000</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -1091,7 +1094,7 @@
         <v/>
       </c>
       <c r="C3" t="str">
-        <v>0.04</v>
+        <v>0.015</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -1146,7 +1149,7 @@
         <v>Guardrails</v>
       </c>
       <c r="B5" t="str">
-        <v>40000</v>
+        <v>250000</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -1161,10 +1164,10 @@
         <v>1.2</v>
       </c>
       <c r="G5" t="str">
+        <v>0.015</v>
+      </c>
+      <c r="H5" t="str">
         <v>0.03</v>
-      </c>
-      <c r="H5" t="str">
-        <v>0.07</v>
       </c>
       <c r="I5" t="str">
         <v>0.1</v>

</xml_diff>